<commit_message>
Backup of existing files
</commit_message>
<xml_diff>
--- a/JobAlert/JobAlert_List.xlsx
+++ b/JobAlert/JobAlert_List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\Projects\Focux\Focux\JobAlert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967C4ACF-89EF-4709-B825-2A4C75251E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FAF65D-B228-4004-91A4-BF9F0D319D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>Index</t>
   </si>
@@ -119,70 +119,88 @@
     <t>class="jobTitle hidden-phone"</t>
   </si>
   <si>
+    <t>Bosch_WerkStudent</t>
+  </si>
+  <si>
+    <t>https://jobs.bosch.com/en/?pages=1&amp;maxDistance=30&amp;searchTerm=werkstudent#</t>
+  </si>
+  <si>
+    <t>Bosch_Thesis</t>
+  </si>
+  <si>
+    <t>https://jobs.bosch.com/en/?pages=1&amp;maxDistance=30&amp;searchTerm=thesis#</t>
+  </si>
+  <si>
+    <t>https://valeo.wd3.myworkdayjobs.com/de-DE/valeo_jobs?locationCountry=dcc5b7608d8644b3a93716604e78e995&amp;workerSubType=1bc7ee912dc9100bd4a8277106db0002</t>
+  </si>
+  <si>
+    <t>https://zeissgroup.wd3.myworkdayjobs.com/External?workerSubType=c2e6b8b5b37f0192a5d38625a300310e</t>
+  </si>
+  <si>
+    <t>Zeiss_WerkStudent</t>
+  </si>
+  <si>
+    <t>data-automation-id="jobTitle"</t>
+  </si>
+  <si>
+    <t>https://zeissgroup.wd3.myworkdayjobs.com/External?q=thesis</t>
+  </si>
+  <si>
+    <t>Zeiss_Thesis</t>
+  </si>
+  <si>
+    <t>Kuka_WerkStudent</t>
+  </si>
+  <si>
+    <t>class="m-results__list-item-headline mod-joblist__headline"</t>
+  </si>
+  <si>
+    <t>https://www.kuka.com/de-de/unternehmen/karriere/stellenangebote?filters=,,566D20CC38E347DCB896F0D8EA6A5F0D|F62D929300DE46BA8932E14D5F5A2894,,409F3B0D508642F5A90FD0E1D679F222|218EE2D37B60454BB1B7FEB342B469F1</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Automotive</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>Robotics</t>
+  </si>
+  <si>
+    <t>class="joboffer_title_text joboffer_box"</t>
+  </si>
+  <si>
+    <t>SEG_Automotive</t>
+  </si>
+  <si>
+    <t>https://career.seg-automotive.com/stellenangebote.html</t>
+  </si>
+  <si>
+    <t>Mbition</t>
+  </si>
+  <si>
+    <t>https://mbition.io/career/</t>
+  </si>
+  <si>
+    <t>class="job-name cpy-28 cpy-b"</t>
+  </si>
+  <si>
     <t>x</t>
   </si>
   <si>
-    <t>Bosch_WerkStudent</t>
-  </si>
-  <si>
-    <t>https://jobs.bosch.com/en/?pages=1&amp;maxDistance=30&amp;searchTerm=werkstudent#</t>
-  </si>
-  <si>
-    <t>Bosch_Thesis</t>
-  </si>
-  <si>
-    <t>https://jobs.bosch.com/en/?pages=1&amp;maxDistance=30&amp;searchTerm=thesis#</t>
-  </si>
-  <si>
-    <t>https://valeo.wd3.myworkdayjobs.com/de-DE/valeo_jobs?locationCountry=dcc5b7608d8644b3a93716604e78e995&amp;workerSubType=1bc7ee912dc9100bd4a8277106db0002</t>
-  </si>
-  <si>
-    <t>https://zeissgroup.wd3.myworkdayjobs.com/External?workerSubType=c2e6b8b5b37f0192a5d38625a300310e</t>
-  </si>
-  <si>
-    <t>Zeiss_WerkStudent</t>
-  </si>
-  <si>
-    <t>data-automation-id="jobTitle"</t>
-  </si>
-  <si>
-    <t>https://zeissgroup.wd3.myworkdayjobs.com/External?q=thesis</t>
-  </si>
-  <si>
-    <t>Zeiss_Thesis</t>
-  </si>
-  <si>
-    <t>Kuka_WerkStudent</t>
-  </si>
-  <si>
-    <t>class="m-results__list-item-headline mod-joblist__headline"</t>
-  </si>
-  <si>
-    <t>https://www.kuka.com/de-de/unternehmen/karriere/stellenangebote?filters=,,566D20CC38E347DCB896F0D8EA6A5F0D|F62D929300DE46BA8932E14D5F5A2894,,409F3B0D508642F5A90FD0E1D679F222|218EE2D37B60454BB1B7FEB342B469F1</t>
-  </si>
-  <si>
-    <t>Domain</t>
-  </si>
-  <si>
-    <t>Automotive</t>
-  </si>
-  <si>
-    <t>IT</t>
-  </si>
-  <si>
-    <t>Robotics</t>
-  </si>
-  <si>
-    <t>class="joboffer_title_text joboffer_box"</t>
-  </si>
-  <si>
-    <t>SEG_Automotive</t>
-  </si>
-  <si>
-    <t>https://career.seg-automotive.com/stellenangebote.html</t>
-  </si>
-  <si>
-    <t>WDebug</t>
+    <t>Messring_Student</t>
+  </si>
+  <si>
+    <t>https://www.messring.de/de/karriere/offene-stellen/?job_position=139</t>
+  </si>
+  <si>
+    <t>itemprop="title name"</t>
+  </si>
+  <si>
+    <t>Debugd</t>
   </si>
 </sst>
 </file>
@@ -569,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="40.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.21875" bestFit="1" customWidth="1"/>
@@ -585,7 +603,7 @@
         <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
         <v>9</v>
@@ -609,7 +627,7 @@
         <v>23</v>
       </c>
       <c r="K1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -620,7 +638,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>5</v>
@@ -646,7 +664,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>6</v>
@@ -672,10 +690,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
         <v>21</v>
@@ -692,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>7</v>
@@ -712,7 +730,7 @@
         <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>25</v>
@@ -722,6 +740,9 @@
       </c>
       <c r="I6">
         <v>2</v>
+      </c>
+      <c r="J6" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -729,13 +750,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
@@ -755,13 +776,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -781,16 +802,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H9" t="s">
-        <v>35</v>
       </c>
       <c r="I9">
         <v>2</v>
@@ -801,16 +822,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I10">
         <v>2</v>
@@ -821,16 +842,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" t="s">
         <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" t="s">
-        <v>39</v>
       </c>
       <c r="I11">
         <v>2</v>
@@ -841,22 +862,59 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="3" t="s">
+      <c r="H12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>47</v>
       </c>
-      <c r="H12" t="s">
-        <v>45</v>
-      </c>
-      <c r="I12">
-        <v>2</v>
-      </c>
-      <c r="J12" t="s">
-        <v>27</v>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -872,6 +930,8 @@
     <hyperlink ref="D10" r:id="rId9" xr:uid="{09266325-9B49-4379-82C8-2035F8F45535}"/>
     <hyperlink ref="D11" r:id="rId10" xr:uid="{0216D34B-2819-46E2-BB42-903120D02667}"/>
     <hyperlink ref="D12" r:id="rId11" xr:uid="{509C0430-4B79-4D15-A29C-B3AB8342C49D}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{8C192A71-60E9-4F7A-86BD-99E6EA51DBBE}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{7159C40D-9747-4F03-8384-BEBE76E6C659}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>